<commit_message>
[Fix] Excel Data 수정
id, name, text / + nameEng, description 등 추가했습니닷
</commit_message>
<xml_diff>
--- a/GameFramework-main/Assets/Resource/GameUnitData.xlsx
+++ b/GameFramework-main/Assets/Resource/GameUnitData.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr codeName="현재_통합_문서" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\사진\바탕 화면\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Team_Project_16\GameFramework-main\Assets\Resource\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910AB40E-5768-47E4-9CB2-23802FE47731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80E901F-26E2-4797-8D16-59D01C10947F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{66E39B16-D752-452C-9266-B1971407CAA6}"/>
+    <workbookView xWindow="4620" yWindow="3915" windowWidth="21600" windowHeight="11835" xr2:uid="{66E39B16-D752-452C-9266-B1971407CAA6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,17 +36,51 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
-  <si>
-    <t>ID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Name</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Text</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+  <si>
+    <t>id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>nameEng</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UnitName</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>power</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>itemType</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>멍멍이</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dog</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>None</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>itemTypeString</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>잘 뛴다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -431,43 +465,66 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E080743-AB47-49F7-9408-727917AC7BB2}">
-  <dimension ref="A1:C6"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
+      <c r="D1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
+      </c>
+      <c r="G2">
+        <v>20</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>